<commit_message>
fix: close migration validation false-pass gaps
</commit_message>
<xml_diff>
--- a/docs/superpowers/specs/2026-04-13-migration-validation.xlsx
+++ b/docs/superpowers/specs/2026-04-13-migration-validation.xlsx
@@ -824,7 +824,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>5-hmdC</t>
+          <t>15N5-8-oxodG</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -834,24 +834,12 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>8.611126060266667</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>438540640</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>344488496.7457034</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>132452176.3030581</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>8.3207268352</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>8.8594375592</v>
-      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>OK</t>
@@ -866,7 +854,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>d3-5-hmdC</t>
+          <t>5-hmdC</t>
         </is>
       </c>
       <c r="C3" s="2" t="n"/>
@@ -950,37 +938,37 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>d3-5-medC</t>
+          <t>8-oxo-Guo</t>
         </is>
       </c>
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>12.62609866611667</v>
+        <v>14.31420593946667</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>202271856</v>
+        <v>399008512</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>151597038.754752</v>
+        <v>310216869.234391</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>56899061.85125972</v>
+        <v>116105791.8024394</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>12.35599852903333</v>
+        <v>14.0007836589</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>12.91424547998333</v>
+        <v>14.64563265331667</v>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NL_FAIL</t>
         </is>
       </c>
     </row>
@@ -992,7 +980,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>N6-HE-dA</t>
+          <t>8-oxodG</t>
         </is>
       </c>
       <c r="C6" s="2" t="n"/>
@@ -1002,24 +990,12 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
-        <v>22.42230274026667</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>409372000</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>324456636.394572</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>139476113.2831667</v>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>22.13236343865</v>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>22.67070759945</v>
-      </c>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t>NL_FAIL</t>
@@ -1034,14 +1010,14 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>d4-N6-2HE-dA</t>
+          <t>N6-HE-dA</t>
         </is>
       </c>
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -1064,7 +1040,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NL_FAIL</t>
         </is>
       </c>
     </row>
@@ -1076,25 +1052,37 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>8-oxodG</t>
+          <t>[13C,15N2]-8-oxo-Guo</t>
         </is>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>14.31420593946667</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>399008512</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>310216869.234391</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>116105791.8024394</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>14.0007836589</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>14.64563265331667</v>
+      </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>NL_FAIL</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1094,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>15N5-8-oxodG</t>
+          <t>d3-5-hmdC</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -1116,12 +1104,24 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="n"/>
+      <c r="F9" s="2" t="n">
+        <v>8.611126060266667</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>438540640</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>344488496.7457034</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>132452176.3030581</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>8.3207268352</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>8.8594375592</v>
+      </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
           <t>OK</t>
@@ -1136,37 +1136,37 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>8-oxo-Guo</t>
+          <t>d3-5-medC</t>
         </is>
       </c>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>14.31420593946667</v>
+        <v>12.62609866611667</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>399008512</v>
+        <v>202271856</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>310216869.234391</v>
+        <v>151597038.754752</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>116105791.8024394</v>
+        <v>56899061.85125972</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>14.0007836589</v>
+        <v>12.35599852903333</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>14.64563265331667</v>
+        <v>12.91424547998333</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>NL_FAIL</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>[13C,15N2]-8-oxo-Guo</t>
+          <t>d4-N6-2HE-dA</t>
         </is>
       </c>
       <c r="C11" s="2" t="n"/>
@@ -1189,22 +1189,22 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>14.31420593946667</v>
+        <v>22.42230274026667</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>399008512</v>
+        <v>409372000</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>310216869.234391</v>
+        <v>324456636.394572</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>116105791.8024394</v>
+        <v>139476113.2831667</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>14.0007836589</v>
+        <v>22.13236343865</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>14.64563265331667</v>
+        <v>22.67070759945</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>5-hmdC</t>
+          <t>15N5-8-oxodG</t>
         </is>
       </c>
       <c r="C12" s="2" t="n"/>
@@ -1231,22 +1231,22 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>8.902873846683333</v>
+        <v>17.56693645441667</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>591372352</v>
+        <v>71953704</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>445196645.9330343</v>
+        <v>63061247.56923112</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>154253783.6772139</v>
+        <v>61383753.67097795</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>8.613854583450001</v>
+        <v>16.53006517171666</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>9.234362482133333</v>
+        <v>17.81591420106667</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>d3-5-hmdC</t>
+          <t>5-hmdC</t>
         </is>
       </c>
       <c r="C13" s="2" t="n"/>
@@ -1346,37 +1346,37 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>d3-5-medC</t>
+          <t>8-oxo-Guo</t>
         </is>
       </c>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>11.42913707813333</v>
+        <v>14.58309869466667</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>279315392</v>
+        <v>397659616</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>163880000.7873313</v>
+        <v>331436394.8090518</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>56255179.26032421</v>
+        <v>129467696.0378032</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>11.18220213521667</v>
+        <v>14.33467711253333</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>11.7402628392</v>
+        <v>14.91445128453333</v>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NL_FAIL</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>N6-HE-dA</t>
+          <t>8-oxodG</t>
         </is>
       </c>
       <c r="C16" s="2" t="n"/>
@@ -1399,26 +1399,26 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>23.35301205706667</v>
+        <v>17.56693645441667</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>396124512</v>
+        <v>71953704</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>346035308.720364</v>
+        <v>63061247.56923112</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>161186738.0376692</v>
+        <v>61383753.67097795</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>23.02058533681667</v>
+        <v>16.53006517171666</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>23.72548893495</v>
+        <v>17.81591420106667</v>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>NO_MS2</t>
+          <t>NL_FAIL</t>
         </is>
       </c>
     </row>
@@ -1430,14 +1430,14 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>d4-N6-2HE-dA</t>
+          <t>N6-HE-dA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NO_MS2</t>
         </is>
       </c>
     </row>
@@ -1472,37 +1472,37 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>8-oxodG</t>
+          <t>[13C,15N2]-8-oxo-Guo</t>
         </is>
       </c>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>17.56693645441667</v>
+        <v>14.58309869466667</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>71953704</v>
+        <v>397659616</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>63061247.56923112</v>
+        <v>331436394.8090518</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>61383753.67097795</v>
+        <v>129467696.0378032</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>16.53006517171666</v>
+        <v>14.33467711253333</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>17.81591420106667</v>
+        <v>14.91445128453333</v>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>NL_FAIL</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>15N5-8-oxodG</t>
+          <t>d3-5-hmdC</t>
         </is>
       </c>
       <c r="C19" s="2" t="n"/>
@@ -1525,22 +1525,22 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>17.56693645441667</v>
+        <v>8.902873846683333</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>71953704</v>
+        <v>591372352</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>63061247.56923112</v>
+        <v>445196645.9330343</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>61383753.67097795</v>
+        <v>154253783.6772139</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>16.53006517171666</v>
+        <v>8.613854583450001</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>17.81591420106667</v>
+        <v>9.234362482133333</v>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
@@ -1556,37 +1556,37 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>8-oxo-Guo</t>
+          <t>d3-5-medC</t>
         </is>
       </c>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>14.58309869466667</v>
+        <v>11.42913707813333</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>397659616</v>
+        <v>279315392</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>331436394.8090518</v>
+        <v>163880000.7873313</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>129467696.0378032</v>
+        <v>56255179.26032421</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>14.33467711253333</v>
+        <v>11.18220213521667</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>14.91445128453333</v>
+        <v>11.7402628392</v>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>NL_FAIL</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>[13C,15N2]-8-oxo-Guo</t>
+          <t>d4-N6-2HE-dA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n"/>
@@ -1609,22 +1609,22 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>14.58309869466667</v>
+        <v>23.35301205706667</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>397659616</v>
+        <v>396124512</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>331436394.8090518</v>
+        <v>346035308.720364</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>129467696.0378032</v>
+        <v>161186738.0376692</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>14.33467711253333</v>
+        <v>23.02058533681667</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>14.91445128453333</v>
+        <v>23.72548893495</v>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>5-hmdC</t>
+          <t>15N5-8-oxodG</t>
         </is>
       </c>
       <c r="C22" s="2" t="n"/>
@@ -1651,22 +1651,22 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>8.626698408233333</v>
+        <v>17.32601291146667</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>847534720</v>
+        <v>48974300</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>583067314.2733066</v>
+        <v>48092153.03710435</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>205860199.4646166</v>
+        <v>29331868.90479133</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>8.336810010366667</v>
+        <v>17.05988601225</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>8.917591178916666</v>
+        <v>17.96421020476667</v>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>d3-5-hmdC</t>
+          <t>5-hmdC</t>
         </is>
       </c>
       <c r="C23" s="2" t="n"/>
@@ -1766,37 +1766,37 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>d3-5-medC</t>
+          <t>8-oxo-Guo</t>
         </is>
       </c>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>12.65148361625</v>
+        <v>14.34101416345</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>314768000</v>
+        <v>435889792</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>237869995.3194584</v>
+        <v>381737098.2552058</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>84872952.71697946</v>
+        <v>177333162.7353577</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>12.37168270851667</v>
+        <v>13.6830715712</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>12.93927853651667</v>
+        <v>14.71385688266667</v>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NL_FAIL</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>N6-HE-dA</t>
+          <t>8-oxodG</t>
         </is>
       </c>
       <c r="C26" s="2" t="n"/>
@@ -1819,22 +1819,22 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>24.10842144613333</v>
+        <v>17.32601291146667</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>235075360</v>
+        <v>48974300</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>195017528.6515848</v>
+        <v>48092153.03710435</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>148670922.6758411</v>
+        <v>29331868.90479133</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>23.40176843943333</v>
+        <v>17.05988601225</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>24.73203024931667</v>
+        <v>17.96421020476667</v>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
@@ -1850,14 +1850,14 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>d4-N6-2HE-dA</t>
+          <t>N6-HE-dA</t>
         </is>
       </c>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NL_FAIL</t>
         </is>
       </c>
     </row>
@@ -1892,37 +1892,37 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>8-oxodG</t>
+          <t>[13C,15N2]-8-oxo-Guo</t>
         </is>
       </c>
       <c r="C28" s="2" t="n"/>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>17.32601291146667</v>
+        <v>14.34101416345</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>48974300</v>
+        <v>435889792</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>48092153.03710435</v>
+        <v>381737098.2552058</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>29331868.90479133</v>
+        <v>177333162.7353577</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>17.05988601225</v>
+        <v>13.6830715712</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>17.96421020476667</v>
+        <v>14.71385688266667</v>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>NL_FAIL</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>15N5-8-oxodG</t>
+          <t>d3-5-hmdC</t>
         </is>
       </c>
       <c r="C29" s="2" t="n"/>
@@ -1945,22 +1945,22 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>17.32601291146667</v>
+        <v>8.626698408233333</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>48974300</v>
+        <v>847534720</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>48092153.03710435</v>
+        <v>583067314.2733066</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>29331868.90479133</v>
+        <v>205860199.4646166</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>17.05988601225</v>
+        <v>8.336810010366667</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>17.96421020476667</v>
+        <v>8.917591178916666</v>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
@@ -1976,37 +1976,37 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>8-oxo-Guo</t>
+          <t>d3-5-medC</t>
         </is>
       </c>
       <c r="C30" s="2" t="n"/>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>14.34101416345</v>
+        <v>12.65148361625</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>435889792</v>
+        <v>314768000</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>381737098.2552058</v>
+        <v>237869995.3194584</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>177333162.7353577</v>
+        <v>84872952.71697946</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>13.6830715712</v>
+        <v>12.37168270851667</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>14.71385688266667</v>
+        <v>12.93927853651667</v>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>NL_FAIL</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>[13C,15N2]-8-oxo-Guo</t>
+          <t>d4-N6-2HE-dA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n"/>
@@ -2029,22 +2029,22 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>14.34101416345</v>
+        <v>24.10842144613333</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>435889792</v>
+        <v>235075360</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>381737098.2552058</v>
+        <v>195017528.6515848</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>177333162.7353577</v>
+        <v>148670922.6758411</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>13.6830715712</v>
+        <v>23.40176843943333</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>14.71385688266667</v>
+        <v>24.73203024931667</v>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
@@ -2060,7 +2060,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>5-hmdC</t>
+          <t>15N5-8-oxodG</t>
         </is>
       </c>
       <c r="C32" s="2" t="n"/>
@@ -2070,12 +2070,24 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
-      <c r="J32" s="2" t="n"/>
-      <c r="K32" s="2" t="n"/>
+      <c r="F32" s="2" t="n">
+        <v>16.19399636908333</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>31972616</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>29939250.87601827</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>6526091.105236913</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>16.07715646106667</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>16.3086088088</v>
+      </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2090,7 +2102,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>d3-5-hmdC</t>
+          <t>5-hmdC</t>
         </is>
       </c>
       <c r="C33" s="2" t="n"/>
@@ -2162,37 +2174,37 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>d3-5-medC</t>
+          <t>8-oxo-Guo</t>
         </is>
       </c>
       <c r="C35" s="2" t="n"/>
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>12.18660909761667</v>
+        <v>14.23085682933333</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>411461600</v>
+        <v>475768864</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>235664483.7230783</v>
+        <v>423294244.4524912</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>81695118.02063768</v>
+        <v>149609232.4977566</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>11.90130822508333</v>
+        <v>13.92439901173333</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>12.46293643441667</v>
+        <v>14.54450614666667</v>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NL_FAIL</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2216,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>N6-HE-dA</t>
+          <t>8-oxodG</t>
         </is>
       </c>
       <c r="C36" s="2" t="n"/>
@@ -2215,26 +2227,26 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>24.0485828256</v>
+        <v>16.19399636908333</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>110899824</v>
+        <v>31972616</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>98934177.13665214</v>
+        <v>29939250.87601827</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>46895015.74778969</v>
+        <v>6526091.105236913</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>23.75762312693333</v>
+        <v>16.07715646106667</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>24.3808995368</v>
+        <v>16.3086088088</v>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>NO_MS2</t>
+          <t>NL_FAIL</t>
         </is>
       </c>
     </row>
@@ -2246,14 +2258,14 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>d4-N6-2HE-dA</t>
+          <t>N6-HE-dA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n"/>
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ND</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -2276,7 +2288,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NO_MS2</t>
         </is>
       </c>
     </row>
@@ -2288,37 +2300,37 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>8-oxodG</t>
+          <t>[13C,15N2]-8-oxo-Guo</t>
         </is>
       </c>
       <c r="C38" s="2" t="n"/>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>16.19399636908333</v>
+        <v>14.23085682933333</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>31972616</v>
+        <v>475768864</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>29939250.87601827</v>
+        <v>423294244.4524912</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>6526091.105236913</v>
+        <v>149609232.4977566</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>16.07715646106667</v>
+        <v>13.92439901173333</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>16.3086088088</v>
+        <v>14.54450614666667</v>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>NL_FAIL</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2342,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>15N5-8-oxodG</t>
+          <t>d3-5-hmdC</t>
         </is>
       </c>
       <c r="C39" s="2" t="n"/>
@@ -2340,24 +2352,12 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="F39" s="2" t="n">
-        <v>16.19399636908333</v>
-      </c>
-      <c r="G39" s="2" t="n">
-        <v>31972616</v>
-      </c>
-      <c r="H39" s="2" t="n">
-        <v>29939250.87601827</v>
-      </c>
-      <c r="I39" s="2" t="n">
-        <v>6526091.105236913</v>
-      </c>
-      <c r="J39" s="2" t="n">
-        <v>16.07715646106667</v>
-      </c>
-      <c r="K39" s="2" t="n">
-        <v>16.3086088088</v>
-      </c>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
           <t>OK</t>
@@ -2372,37 +2372,37 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>8-oxo-Guo</t>
+          <t>d3-5-medC</t>
         </is>
       </c>
       <c r="C40" s="2" t="n"/>
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>14.23085682933333</v>
+        <v>12.18660909761667</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>475768864</v>
+        <v>411461600</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>423294244.4524912</v>
+        <v>235664483.7230783</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>149609232.4977566</v>
+        <v>81695118.02063768</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>13.92439901173333</v>
+        <v>11.90130822508333</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>14.54450614666667</v>
+        <v>12.46293643441667</v>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>NL_FAIL</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>[13C,15N2]-8-oxo-Guo</t>
+          <t>d4-N6-2HE-dA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n"/>
@@ -2425,22 +2425,22 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>14.23085682933333</v>
+        <v>24.0485828256</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>475768864</v>
+        <v>110899824</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>423294244.4524912</v>
+        <v>98934177.13665214</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>149609232.4977566</v>
+        <v>46895015.74778969</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>13.92439901173333</v>
+        <v>23.75762312693333</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>14.54450614666667</v>
+        <v>24.3808995368</v>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>

</xml_diff>